<commit_message>
Add the style A/B sheet, with the rows style never reached greyed out
The generated columns mislead on their own. Style reached 5 of the 12
questions; the other 7 are byte-identical because they scored below the 0.60
retrieval floor, so a reviewer comparing them is comparing nothing. Those
rows are greyed, and a reviewed column reads each flagged row rather than
counting its figures -- of the flags, one is a real loss (the Rs 45,000
emergency-fund anchor), the rest are reformatting or trimmed asides.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/style-comparison-final.xlsx
+++ b/docs/style-comparison-final.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +37,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +59,16 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -81,6 +95,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -460,6 +481,8 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,17 +541,27 @@
           <t>Which reads better?</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Did style apply?</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed (read, not counted)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>मेरी बेटी 5 साल की है, उसके लिए कौन सी सरकारी योजना अच्छी है?</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>आपकी बेटी के लिए **सुकन्या समृद्धि योजना (Sukanya Samriddhi Yojana)** सबसे अच्छा विकल्प है।
 यह योजना विशेष रूप से बालिकाओं की शिक्षा और शादी के भविष्य के लिए बनाई गई है:
@@ -538,7 +571,7 @@
 **ध्यान दें:** छोटी बचत योजनाओं की दरें हर तिमाही (3 महीने) में बदल सकती हैं। कृपया बैंक या डाकघर से नवीनतम जानकारी पुष्टि कर लें।</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>आपकी बेटी के लिए **सुकन्या समृद्धि योजना (Sukanya Samriddhi Yojana)** सबसे अच्छा विकल्प है।
 यह योजना विशेष रूप से बालिकाओं की शिक्षा और शादी के भविष्य के लिए बनाई गई है:
@@ -548,82 +581,102 @@
 **ध्यान दें:** छोटी बचत योजनाओं की दरें हर तिमाही (3 महीने) में बदल सकती हैं। कृपया बैंक या डाकघर से नवीनतम जानकारी पुष्टि कर लें।</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="n">
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="6" t="n">
         <v>9.4</v>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr"/>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>no — below 0.60 floor</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>IDENTICAL answers. Nothing to compare on this row.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>1 लाख रुपये 1 साल की FD में रखूं तो मैच्योरिटी पर कितना मिलेगा?</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>1 लाख रुपये की 1 साल की FD मैच्योर होने पर आपको **₹1,06,398.02** मिलेंगे। इसमें ₹6,398.02 ब्याज शामिल है।
 ये रेट SBI के 15 दिसंबर 2025 से लागू हो रहे हैं। ध्यान रखें कि FD पर जो ब्याज मिलता है, वो आपके टैक्स स्लैब के हिसाब से टैबेबल होता है।</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>1 लाख रुपये की 1 साल की FD मैच्योर होने पर आपको **₹1,06,398.02** मिलेंगे। इसमें ₹6,398.02 ब्याज शामिल है।
 ये रेट SBI के 15 दिसंबर 2025 से लागू हो रहे हैं। ध्यान रखें कि FD पर जो ब्याज मिलता है, वो आपके टैक्स स्लैब के हिसाब से टैबेबल होता है।</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>india.get_fd_rate, money.fd_maturity</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>india.get_fd_rate, money.fd_maturity</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="n">
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="n">
         <v>9.6</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="6" t="n">
         <v>10.4</v>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>no — below 0.60 floor</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>IDENTICAL answers. Nothing to compare on this row.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -674,68 +727,88 @@
         <v>8</v>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>style applied</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>GAINED — answer nearly doubled (215→419) and states the rate correctly. Flagged figures are reformatting, not loss.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>मैं महीने के 15000 कमाता हूँ, बैंक से सस्ता बीमा कौन सा मिलेगा?</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>सबसे सस्ता बीमा **प्रधानमंत्री सुरक्षा बीमा योजना (PMSBY)** है, जिसका प्रीमियम सिर्फ ₹20 प्रति वर्ष है।
 ध्यान दें: PMSBY में केवल **दुर्घटना से मृत्यु या अपंगता** की कवरेज होती है, बीमारी से मृत्यु नहीं।
 अगर आपको बीमारी सहित किसी भी कारण से मृत्यु का खतरा है, तो **प्रधानमंत्री जीवन ज्योति बीमा योजना (PMJJBY)** लें, जिसका प्रीमियम ₹436 प्रति वर्ष है।</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>सबसे सस्ता बीमा **प्रधानमंत्री सुरक्षा बीमा योजना (PMSBY)** है, जिसका प्रीमियम सिर्फ ₹20 प्रति वर्ष है।
 ध्यान दें: PMSBY में केवल **दुर्घटना से मृत्यु या अपंगता** की कवरेज होती है, बीमारी से मृत्यु नहीं।
 अगर आपको बीमारी सहित किसी भी कारण से मृत्यु का खतरा है, तो **प्रधानमंत्री जीवन ज्योति बीमा योजना (PMJJBY)** लें, जिसका प्रीमियम ₹436 प्रति वर्ष है।</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="n">
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>8.4</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="6" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>no — below 0.60 floor</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>IDENTICAL answers. Nothing to compare on this row.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>PPF क्या है और इसमें कितना ब्याज मिलता है?</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>PPF (Public Provident Fund) एक सरकारी द्वारा समर्थित लॉन्ग-टर्म बचत योजना है। इसमें आप न्यूनतम 1 वर्ष के लिए निवेश करते हैं, लेकिन पूरा टर्म 15 साल होता है।
 इस पर **7.1%** की दर से ब्याज मिलता है। यह दर Ministry of Finance द्वारा हर क्वार्टर (3 महीने) में अपडेट की जाती है।
@@ -745,7 +818,7 @@
 - **Note:** चूंकि छोटी बचत दरें हर क्वार्टर बदल सकती हैं, इसलिए नवीनतम जानकारी के लिए nsiindia.gov.in या अपने बैंक से पुष्टि कर लें।</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>PPF (Public Provident Fund) एक सरकारी द्वारा समर्थित लॉन्ग-टर्म बचत योजना है। इसमें आप न्यूनतम 1 वर्ष के लिए निवेश करते हैं, लेकिन पूरा टर्म 15 साल होता है।
 इस पर **7.1%** की दर से ब्याज मिलता है। यह दर Ministry of Finance द्वारा हर क्वार्टर (3 महीने) में अपडेट की जाती है।
@@ -755,44 +828,54 @@
 - **Note:** चूंकि छोटी बचत दरें हर क्वार्टर बदल सकती हैं, इसलिए नवीनतम जानकारी के लिए nsiindia.gov.in या अपने बैंक से पुष्टि कर लें।</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="n">
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="6" t="n">
         <v>9.5</v>
       </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>no — below 0.60 floor</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>IDENTICAL answers. Nothing to compare on this row.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>मैं 62 साल का हूँ, हर महीने इनकम के लिए कौन सा विकल्प अच्छा है?</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>62 साल की उम्र में आप सीनियर सिटीजन के तहत बेहतर ब्याज दरें पा सकते हैं। यहाँ कुछ विकल्प दिए गए हैं:
 1. **बैंक FD (सावधि जमा):** SBI जैसे बैंकों में 12 महीने की FD पर सीनियर सिटीजन को 6.75% प्रति वर्ष मिलते हैं। यह दर 15 दिसंबर 2025 से लागू है।
@@ -801,7 +884,7 @@
 **ध्यान दें:** सरकारी स्कीमों की दरें हर तिमाही (3 महीने) में बदल सकती हैं। कृपया किसी भी निवेश से पहले अपनी नजदीकी बैंक या पोस्ट ऑफिस से पुष्टि कर लें।</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>62 साल की उम्र में आप सीनियर सिटीजन के तहत बेहतर ब्याज दरें पा सकते हैं। यहाँ कुछ विकल्प दिए गए हैं:
 1. **बैंक FD (सावधि जमा):** SBI जैसे बैंकों में 12 महीने की FD पर सीनियर सिटीजन को 6.75% प्रति वर्ष मिलते हैं। यह दर 15 दिसंबर 2025 से लागू है।
@@ -810,33 +893,43 @@
 **ध्यान दें:** सरकारी स्कीमों की दरें हर तिमाही (3 महीने) में बदल सकती हैं। कृपया किसी भी निवेश से पहले अपनी नजदीकी बैंक या पोस्ट ऑफिस से पुष्टि कर लें।</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>india.get_fd_rate, india.get_scheme_details</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>india.get_fd_rate, india.get_scheme_details</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
         <v>14.9</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="6" t="n">
         <v>15.7</v>
       </c>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>no — below 0.60 floor</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>IDENTICAL answers. Nothing to compare on this row.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -908,57 +1001,77 @@
         <v>11</v>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>style applied</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>CLEAN — 783→787 chars, nothing lost.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>अगर बैंक डूब जाए तो मेरा कितना पैसा सुरक्षित है?</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>अगर आपका बैंक डूब जाता है, तो डिपॉजिट इन्श्योरेंस एंड गारंटी कॉर्पोरेशन ऑफ इंडिया (DICGC) के तहत **₹5,00,000** तक का पैसा सुरक्षित होता है।
 यह राशि आपके मूल धन और उस पर जुड़े ब्याज दोनों को मिलकर ढकती है। यह कवरेज हर बैंक में अलग-अलग शाखाओं में रखी गई सारी जमा राशियों को जोड़कर लागू होता है, न कि प्रति व्यक्ति या प्रति खाता।
 स्रोत: RBI FAQ — Deposit Insurance (DICGC)</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>अगर आपका बैंक डूब जाता है, तो डिपॉजिट इन्श्योरेंस एंड गारंटी कॉर्पोरेशन ऑफ इंडिया (DICGC) के तहत **₹5,00,000** तक का पैसा सुरक्षित होता है।
 यह राशि आपके मूल धन और उस पर जुड़े ब्याज दोनों को मिलकर ढकती है। यह कवरेज हर बैंक में अलग-अलग शाखाओं में रखी गई सारी जमा राशियों को जोड़कर लागू होता है, न कि प्रति व्यक्ति या प्रति खाता।
 स्रोत: RBI FAQ — Deposit Insurance (DICGC)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>docs.search</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>docs.search</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="n">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n">
         <v>10.8</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="6" t="n">
         <v>11.6</v>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>no — below 0.60 floor</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>IDENTICAL answers. Nothing to compare on this row.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1019,6 +1132,16 @@
         <v>14.2</v>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>style applied</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>MINOR — shorter (993→781). Core answer intact.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1076,6 +1199,16 @@
         <v>9.800000000000001</v>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>style applied</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>WATCH — emergency-fund advice survives, but the ₹45,000 anchor is gone. The one loss that still matters.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1125,17 +1258,27 @@
         <v>8.1</v>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>style applied</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>CLEAN — 230→263 chars, nothing lost.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>बुढ़ापे के लिए पेंशन का क्या इंतज़ाम करूं?</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>बुढ़ापे की सुरक्षा के लिए सरकार की कई स्कीमें हैं। आप अपनी उम्र और जरूरत के हिसाब से चुन सकते हैं:
 1. अटल पेंशन योजना (APY): यह सीधे बुढ़ापे के लिए है। आप 60 साल की उम्र तक माहिर ₹1,000 से ₹5,000 का पेंशन चुन सकते हैं। इसका योगदान आपकी वर्तमान उम्र पर निर्भर करता है, इसलिए सटीक राशि जानने के लिए अपने बैंक से संपर्क करें।
@@ -1145,7 +1288,7 @@
 5. पॉस्ट ऑफिस मंथली इनकम स्कीम (POMIS): यदि आपको नियमित मासिक आय चाहिए, तो यह स्कीम उपयुक्त हो सकती है।</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>बुढ़ापे की सुरक्षा के लिए सरकार की कई स्कीमें हैं। आप अपनी उम्र और जरूरत के हिसाब से चुन सकते हैं:
 1. अटल पेंशन योजना (APY): यह सीधे बुढ़ापे के लिए है। आप 60 साल की उम्र तक माहिर ₹1,000 से ₹5,000 का पेंशन चुन सकते हैं। इसका योगदान आपकी वर्तमान उम्र पर निर्भर करता है, इसलिए सटीक राशि जानने के लिए अपने बैंक से संपर्क करें।
@@ -1155,33 +1298,43 @@
 5. पॉस्ट ऑफिस मंथली इनकम स्कीम (POMIS): यदि आपको नियमित मासिक आय चाहिए, तो यह स्कीम उपयुक्त हो सकती है।</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>india.get_scheme_details</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n">
         <v>10.4</v>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="J13" s="6" t="n">
         <v>11.3</v>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>no — below 0.60 floor</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>IDENTICAL answers. Nothing to compare on this row.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1194,102 +1347,185 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="104" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>What this compares</t>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>FinGuru — Hindi style A/B</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Each question was answered twice by the same agent in one run.</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WITHOUT style = today's behaviour. WITH style = vernacular examples added to the prompt.</t>
+          <t>Each question was answered twice by the same agent, in one run.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WITHOUT style = current shipped behaviour. WITH style = vernacular examples added to the prompt.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>The only question for a reviewer</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Does the WITH column read more like how a person would explain it — while saying the same thing?</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>READ THIS FIRST</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fill in 'Which reads better?' with: without / with / same.</t>
+          <t>Style only reached 5 of the 12 questions. The other 7 are byte-identical and are greyed out —</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>skip them. Retrieval requires a similarity of 0.60 and the other 7 scored below it, because the</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Two columns to check first</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>corpus (61 videos) covers gold loans, app walkthroughs and account opening, and barely touches</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Same tools? — the runs each look things up separately. 'NO' means the answers differ for</t>
+          <t>schemes, pensions, senior citizens or insurance. That is a corpus gap, not a prompt problem.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    reasons unrelated to style, so that row is not a fair comparison.</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Numbers preserved? — every figure in the WITHOUT answer, checked against the WITH answer.</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>THE ONE QUESTION FOR A REVIEWER</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'NO' is a defect, not a style choice. Style may change wording and nothing else.</t>
+          <t>On the 5 rows where style applied: does the WITH column read more like how a person would</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>actually explain it, while saying the same thing? Fill in 'Which reads better?' with</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Red cells mean look here.</t>
+          <t>without / with / same. A Hindi speaker's judgement is the only thing that settles this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>THE SAFETY COLUMNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Same tools? — 12/12. Both versions called identical tools, so grounding is unaffected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Numbers preserved? — automated, and it cannot tell a trimmed aside from a dropped fact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    It flags reformatting too: '₹2,00,000' rewritten as '₹2 लाख' is the same sum said the way</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    a person says it, which is the point of the layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Reviewed — a read of each flagged row in full. Of the flags, ONE is a real loss (row 10,</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    the ₹45,000 emergency-fund anchor). No answer was ever wrong; nothing was invented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ALREADY FIXED, VISIBLE IN THIS RUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>An earlier run closed one answer with 'or you'll end up a servant of the bank' — invented by</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>the model, not present anywhere in the corpus, because the register it copies ends on a punchy</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>line. A guard was added; no sign-off appears in this run.</t>
         </is>
       </c>
     </row>

</xml_diff>